<commit_message>
added extra data on participants and valid_tags for poc8 and poc9
</commit_message>
<xml_diff>
--- a/data/embrace_plus/participants_extra_data/participant_data_periods.xlsx
+++ b/data/embrace_plus/participants_extra_data/participant_data_periods.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workdir\ptsd-attack-prediction\data\embrace_plus\participants_extra_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FCF933CF-D5A8-4196-8D88-C534219F8FF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{135F3900-34AE-4149-B8E7-C90BBF943D7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E4202787-E82A-43CD-A074-A1D79704F9D5}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{E4202787-E82A-43CD-A074-A1D79704F9D5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>nickName</t>
   </si>
@@ -80,12 +81,21 @@
   </si>
   <si>
     <t>POC11</t>
+  </si>
+  <si>
+    <t>POC12</t>
+  </si>
+  <si>
+    <t>POC13</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="[$-1010409]d/m/yyyy\ h:mm;@"/>
+  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -209,20 +219,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="2" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
@@ -238,16 +236,22 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="22" fontId="2" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="22" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="22" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
@@ -584,134 +588,154 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49A5CC8A-7045-4A68-A678-5596C0E31FE3}">
-  <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.59765625" style="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.09765625" style="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.3984375" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="8.796875" style="8"/>
+    <col min="1" max="1" width="9.625" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.125" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.125" style="4" customWidth="1"/>
+    <col min="4" max="16384" width="8.75" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="28.2" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
+    <row r="2" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="10">
-        <v>45746.677083333336</v>
-      </c>
-      <c r="C2" s="1">
-        <v>45777</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="11" t="s">
+      <c r="B2" s="7">
+        <v>45746.669444444444</v>
+      </c>
+      <c r="C2" s="8">
+        <v>45776.736111111109</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="12">
-        <v>45756.604166666664</v>
-      </c>
-      <c r="C3" s="2">
-        <v>45785</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="9" t="s">
+      <c r="B3" s="9">
+        <v>45756.602777777778</v>
+      </c>
+      <c r="C3" s="10">
+        <v>45785.8125</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="7">
         <v>45771.486111111109</v>
       </c>
-      <c r="C4" s="1">
-        <v>45800</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="11" t="s">
+      <c r="C4" s="8">
+        <v>45800.431250000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="13">
-        <v>45772.625</v>
-      </c>
-      <c r="C5" s="2">
-        <v>45803</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="9" t="s">
+      <c r="B5" s="11">
+        <v>45774.625</v>
+      </c>
+      <c r="C5" s="10">
+        <v>45803.600694444445</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="7">
         <v>45791.49722222222</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="8">
         <v>45825</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="11" t="s">
+    <row r="7" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
         <v>8</v>
       </c>
       <c r="B7" s="10">
         <v>45887.520833333336</v>
       </c>
-      <c r="C7" s="3"/>
-    </row>
-    <row r="8" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="9" t="s">
+      <c r="C7" s="10"/>
+    </row>
+    <row r="8" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="10"/>
-      <c r="C8" s="4"/>
-    </row>
-    <row r="9" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="11" t="s">
+      <c r="B8" s="7"/>
+      <c r="C8" s="8"/>
+    </row>
+    <row r="9" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="12">
+      <c r="B9" s="9">
         <v>45848.618055555555</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="10">
         <v>45879</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="9" t="s">
+    <row r="10" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="10">
+      <c r="B10" s="7">
         <v>45869.552083333336</v>
       </c>
-      <c r="C10" s="4"/>
-    </row>
-    <row r="11" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="11" t="s">
+      <c r="C10" s="7">
+        <v>45898.416666666664</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="12">
+      <c r="B11" s="9">
         <v>45872.45</v>
       </c>
-      <c r="C11" s="3"/>
-    </row>
-    <row r="12" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="9" t="s">
+      <c r="C11" s="10"/>
+    </row>
+    <row r="12" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="10">
+      <c r="B12" s="7">
         <v>45883.583333333336</v>
       </c>
-      <c r="C12" s="4"/>
+      <c r="C12" s="8"/>
+    </row>
+    <row r="13" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="10">
+        <v>45897.5625</v>
+      </c>
+      <c r="C13" s="10"/>
+    </row>
+    <row r="14" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" s="7">
+        <v>45900.5</v>
+      </c>
+      <c r="C14" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -725,7 +749,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18919ACF-1A96-4FF3-833A-8ACDADB9A796}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
@@ -738,7 +762,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C54AADA-7438-4E9F-9B79-4BD29E6DACEE}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>

</xml_diff>

<commit_message>
Added tags to poc10-14
</commit_message>
<xml_diff>
--- a/data/embrace_plus/participants_extra_data/participant_data_periods.xlsx
+++ b/data/embrace_plus/participants_extra_data/participant_data_periods.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workdir\ptsd-attack-prediction\data\embrace_plus\participants_extra_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{135F3900-34AE-4149-B8E7-C90BBF943D7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFD2F7F8-A2D3-405E-BE14-8007040801F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{E4202787-E82A-43CD-A074-A1D79704F9D5}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E4202787-E82A-43CD-A074-A1D79704F9D5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,6 @@
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>nickName</t>
   </si>
@@ -87,6 +86,9 @@
   </si>
   <si>
     <t>POC13</t>
+  </si>
+  <si>
+    <t>POC14</t>
   </si>
 </sst>
 </file>
@@ -119,7 +121,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -135,6 +137,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFCAEDFB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -219,7 +227,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
@@ -253,6 +261,12 @@
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -588,7 +602,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49A5CC8A-7045-4A68-A678-5596C0E31FE3}">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.625" style="4" bestFit="1" customWidth="1"/>
@@ -670,14 +684,20 @@
       <c r="B7" s="10">
         <v>45887.520833333336</v>
       </c>
-      <c r="C7" s="10"/>
+      <c r="C7" s="10">
+        <v>45925.5</v>
+      </c>
     </row>
     <row r="8" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="8"/>
+      <c r="B8" s="13">
+        <v>45848.465277777781</v>
+      </c>
+      <c r="C8" s="13">
+        <v>45851.395833333336</v>
+      </c>
     </row>
     <row r="9" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
@@ -698,7 +718,7 @@
         <v>45869.552083333336</v>
       </c>
       <c r="C10" s="7">
-        <v>45898.416666666664</v>
+        <v>45897.416666666664</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
@@ -708,7 +728,9 @@
       <c r="B11" s="9">
         <v>45872.45</v>
       </c>
-      <c r="C11" s="10"/>
+      <c r="C11" s="9">
+        <v>45901.5</v>
+      </c>
     </row>
     <row r="12" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
@@ -717,16 +739,20 @@
       <c r="B12" s="7">
         <v>45883.583333333336</v>
       </c>
-      <c r="C12" s="8"/>
+      <c r="C12" s="7">
+        <v>45921.541666666664</v>
+      </c>
     </row>
     <row r="13" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>14</v>
       </c>
       <c r="B13" s="10">
-        <v>45897.5625</v>
-      </c>
-      <c r="C13" s="10"/>
+        <v>45897.583333333336</v>
+      </c>
+      <c r="C13" s="10">
+        <v>45925.416666666664</v>
+      </c>
     </row>
     <row r="14" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
@@ -735,7 +761,18 @@
       <c r="B14" s="7">
         <v>45900.5</v>
       </c>
-      <c r="C14" s="8"/>
+      <c r="C14" s="7">
+        <v>45925.5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="10">
+        <v>45946.541666666664</v>
+      </c>
+      <c r="C15" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Adding tags modification using anomaly
</commit_message>
<xml_diff>
--- a/data/embrace_plus/participants_extra_data/participant_data_periods.xlsx
+++ b/data/embrace_plus/participants_extra_data/participant_data_periods.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workdir\ptsd-attack-prediction\data\embrace_plus\participants_extra_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFD2F7F8-A2D3-405E-BE14-8007040801F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E983286-6E93-4B73-900A-38C3F7788CF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E4202787-E82A-43CD-A074-A1D79704F9D5}"/>
+    <workbookView xWindow="7812" yWindow="0" windowWidth="23004" windowHeight="16656" xr2:uid="{E4202787-E82A-43CD-A074-A1D79704F9D5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
   <si>
     <t>nickName</t>
   </si>
@@ -89,6 +89,72 @@
   </si>
   <si>
     <t>POC14</t>
+  </si>
+  <si>
+    <t>POC15</t>
+  </si>
+  <si>
+    <t>POC16</t>
+  </si>
+  <si>
+    <t>POC17</t>
+  </si>
+  <si>
+    <t>?</t>
+  </si>
+  <si>
+    <t>user_id</t>
+  </si>
+  <si>
+    <t>TRAIL003</t>
+  </si>
+  <si>
+    <t>TRAIL002</t>
+  </si>
+  <si>
+    <t>TRAIL001</t>
+  </si>
+  <si>
+    <t>TRAIL04</t>
+  </si>
+  <si>
+    <t>TRAIL005</t>
+  </si>
+  <si>
+    <t>TRAIL006</t>
+  </si>
+  <si>
+    <t>TRAIL007</t>
+  </si>
+  <si>
+    <t>TRAIL008</t>
+  </si>
+  <si>
+    <t>TRAIL009</t>
+  </si>
+  <si>
+    <t>TRAIL10</t>
+  </si>
+  <si>
+    <t>TRAIL011</t>
+  </si>
+  <si>
+    <t>TRAIL012</t>
+  </si>
+  <si>
+    <t>TRAIL013</t>
+  </si>
+  <si>
+    <t>TRAIL014</t>
+  </si>
+  <si>
+    <t>TRAIL015</t>
+  </si>
+  <si>
+    <t>TRAIL016</t>
+  </si>
+  <si>
+    <t>TRAIL017</t>
   </si>
 </sst>
 </file>
@@ -147,49 +213,12 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="9">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF0F9ED5"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF0F9ED5"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF0F9ED5"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="FF0F9ED5"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF0F9ED5"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF0F9ED5"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color rgb="FF0F9ED5"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF0F9ED5"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -223,56 +252,298 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF0F9ED5"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF0F9ED5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF0F9ED5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF0F9ED5"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF0F9ED5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF60CAF3"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF60CAF3"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="7">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF0F9ED5"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="[$-1010409]d/m/yyyy\ h:mm;@"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FF60CAF3"/>
+        </left>
+        <right/>
+        <top/>
+        <bottom style="medium">
+          <color rgb="FF60CAF3"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="[$-1010409]d/m/yyyy\ h:mm;@"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FF60CAF3"/>
+        </left>
+        <right/>
+        <top/>
+        <bottom style="medium">
+          <color rgb="FF60CAF3"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFCAEDFB"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="medium">
+          <color rgb="FF60CAF3"/>
+        </right>
+        <top/>
+        <bottom style="medium">
+          <color rgb="FF60CAF3"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFCAEDFB"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="medium">
+          <color rgb="FF60CAF3"/>
+        </right>
+        <top/>
+        <bottom style="medium">
+          <color rgb="FF60CAF3"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color rgb="FF0F9ED5"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color rgb="FF0F9ED5"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF60CAF3"/>
+        </bottom>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -283,6 +554,19 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B04E6431-8301-41CD-BD3D-3C79231195D9}" name="Table2" displayName="Table2" ref="A1:D18" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="5" tableBorderDxfId="6">
+  <autoFilter ref="A1:D18" xr:uid="{B04E6431-8301-41CD-BD3D-3C79231195D9}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{26981ACF-EE35-469D-8814-A0FA8B1DE0BB}" name="nickName" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{822C130D-17C5-42DB-8B39-BCA5289C13C6}" name="user_id" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{AB29FB62-FF0A-4119-8AAA-05C00086156E}" name="trial_starting_date" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{879DC26B-09EC-4BD7-B4A2-B2AEF4270BFE}" name="trial_ending_date" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -602,191 +886,285 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49A5CC8A-7045-4A68-A678-5596C0E31FE3}">
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr defaultColWidth="8.69921875" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.625" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.125" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.125" style="4" customWidth="1"/>
-    <col min="4" max="16384" width="8.75" style="4"/>
+    <col min="1" max="1" width="13.59765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.3984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.69921875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.09765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="8.69921875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="14" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+    <row r="2" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="7">
+      <c r="B2" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="4">
         <v>45746.669444444444</v>
       </c>
-      <c r="C2" s="8">
+      <c r="D2" s="5">
         <v>45776.736111111109</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+    <row r="3" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="6">
         <v>45756.602777777778</v>
       </c>
-      <c r="C3" s="10">
+      <c r="D3" s="7">
         <v>45785.8125</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
+    <row r="4" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="7">
+      <c r="B4" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="4">
         <v>45771.486111111109</v>
       </c>
-      <c r="C4" s="8">
+      <c r="D4" s="5">
         <v>45800.431250000001</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+    <row r="5" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="11">
+      <c r="B5" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="8">
         <v>45774.625</v>
       </c>
-      <c r="C5" s="10">
+      <c r="D5" s="7">
         <v>45803.600694444445</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+    <row r="6" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="8">
         <v>45791.49722222222</v>
       </c>
-      <c r="C6" s="8">
+      <c r="D6" s="5">
         <v>45825</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+    <row r="7" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="8">
         <v>45887.520833333336</v>
       </c>
-      <c r="C7" s="10">
+      <c r="D7" s="7">
         <v>45925.5</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="12" t="s">
+    <row r="8" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="13">
+      <c r="B8" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="10">
         <v>45848.465277777781</v>
       </c>
-      <c r="C8" s="13">
+      <c r="D8" s="10">
         <v>45851.395833333336</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
+    <row r="9" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="9">
+      <c r="B9" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="6">
         <v>45848.618055555555</v>
       </c>
-      <c r="C9" s="10">
+      <c r="D9" s="7">
         <v>45879</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
+    <row r="10" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="7">
+      <c r="B10" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="4">
         <v>45869.552083333336</v>
       </c>
-      <c r="C10" s="7">
+      <c r="D10" s="4">
         <v>45897.416666666664</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
+    <row r="11" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="9">
+      <c r="B11" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" s="6">
         <v>45872.45</v>
       </c>
-      <c r="C11" s="9">
+      <c r="D11" s="6">
         <v>45901.5</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
+    <row r="12" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="7">
+      <c r="B12" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="4">
         <v>45883.583333333336</v>
       </c>
-      <c r="C12" s="7">
+      <c r="D12" s="4">
         <v>45921.541666666664</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
+    <row r="13" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C13" s="7">
         <v>45897.583333333336</v>
       </c>
-      <c r="C13" s="10">
+      <c r="D13" s="7">
         <v>45925.416666666664</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
+    <row r="14" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="7">
-        <v>45900.5</v>
-      </c>
-      <c r="C14" s="7">
+      <c r="B14" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" s="4">
+        <v>45900.541666666664</v>
+      </c>
+      <c r="D14" s="4">
         <v>45925.5</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
+    <row r="15" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="10">
+      <c r="B15" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15" s="7">
         <v>45946.541666666664</v>
       </c>
-      <c r="C15" s="10"/>
+      <c r="D15" s="7">
+        <v>45985.395833333336</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C16" s="7">
+        <v>45971.463888888888</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C17" s="7">
+        <v>45985.384027777778</v>
+      </c>
+      <c r="D17" s="7">
+        <v>46033.5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" s="16" t="s">
+        <v>38</v>
+      </c>
+      <c r="C18" s="17">
+        <v>45998.354166666664</v>
+      </c>
+      <c r="D18" s="17">
+        <v>46033.4375</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"Calibri"&amp;10&amp;K008000 OFFICIAL&amp;1#_x000D_</oddHeader>
     <oddFooter>&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K008000 OFFICIAL</oddFooter>
   </headerFooter>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18919ACF-1A96-4FF3-833A-8ACDADB9A796}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
@@ -799,7 +1177,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C54AADA-7438-4E9F-9B79-4BD29E6DACEE}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>

</xml_diff>

<commit_message>
Updated tags according to new final report on participants
</commit_message>
<xml_diff>
--- a/data/embrace_plus/participants_extra_data/participant_data_periods.xlsx
+++ b/data/embrace_plus/participants_extra_data/participant_data_periods.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workdir\ptsd-attack-prediction\data\embrace_plus\participants_extra_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{980A8BC6-1D5E-4153-B3B7-4BF605E2BE31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E864BEC-8CFC-4FE5-AC3F-4A69B0F9510E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7812" yWindow="0" windowWidth="23004" windowHeight="16656" xr2:uid="{E4202787-E82A-43CD-A074-A1D79704F9D5}"/>
+    <workbookView xWindow="-30828" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{E4202787-E82A-43CD-A074-A1D79704F9D5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1114,7 +1114,7 @@
         <v>45971.463888888888</v>
       </c>
       <c r="D16" s="17">
-        <v>46006.354166666664</v>
+        <v>45998.354166666664</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">

</xml_diff>